<commit_message>
Updated Streamlit app: new files, code changes, and data added
</commit_message>
<xml_diff>
--- a/GT_DATA_122_merged_filled.xlsx
+++ b/GT_DATA_122_merged_filled.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Harshit\kenya_dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{228B9070-857B-48D1-A566-1E62602DBBC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01B93C7F-B53E-4FCB-9E89-A387906F2BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2012,7 +2012,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>17</v>
       </c>
@@ -2065,7 +2065,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -2436,7 +2436,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -2489,7 +2489,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>140</v>
       </c>
@@ -2648,7 +2648,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>140</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>41</v>
       </c>
@@ -2954,7 +2954,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>41</v>
       </c>
@@ -3060,7 +3060,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>45</v>
       </c>
@@ -3219,7 +3219,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>45</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>0.14323814186795089</v>
       </c>
       <c r="J51">
-        <v>-4.0468103472254002</v>
+        <v>-4.7234722539999998</v>
       </c>
       <c r="K51" t="s">
         <v>62</v>
@@ -3643,7 +3643,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>17</v>
       </c>
@@ -3778,7 +3778,7 @@
         <v>1.58655824885682</v>
       </c>
       <c r="J56">
-        <v>-4.0468103472254002</v>
+        <v>-2.0468103472253998</v>
       </c>
       <c r="K56" t="s">
         <v>35</v>
@@ -3802,7 +3802,7 @@
         <v>0.90978512675522105</v>
       </c>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>34</v>
       </c>
@@ -3990,7 +3990,7 @@
         <v>-8.9965602273005055E-2</v>
       </c>
       <c r="J60">
-        <v>-4.0468103472254002</v>
+        <v>-4.8681029999999996</v>
       </c>
       <c r="K60" t="s">
         <v>38</v>
@@ -4385,7 +4385,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>140</v>
       </c>
@@ -4467,7 +4467,7 @@
         <v>0.74078304227831238</v>
       </c>
       <c r="J69">
-        <v>-4.0468103472254002</v>
+        <v>-1.0673472254</v>
       </c>
       <c r="K69" t="s">
         <v>28</v>
@@ -4491,7 +4491,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>41</v>
       </c>
@@ -4573,7 +4573,7 @@
         <v>0.26226205021275978</v>
       </c>
       <c r="J71">
-        <v>-4.0468103472254002</v>
+        <v>-7.0468103472254002</v>
       </c>
       <c r="K71" t="s">
         <v>62</v>
@@ -4597,7 +4597,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>45</v>
       </c>
@@ -4756,7 +4756,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>34</v>
       </c>
@@ -4809,7 +4809,7 @@
         <v>0.21300635211888899</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>17</v>
       </c>
@@ -4862,7 +4862,7 @@
         <v>0.33574615975324601</v>
       </c>
     </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>41</v>
       </c>
@@ -4915,7 +4915,7 @@
         <v>0.50738586856954204</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>140</v>
       </c>
@@ -4968,7 +4968,7 @@
         <v>0.152982473655638</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>45</v>
       </c>
@@ -5021,7 +5021,7 @@
         <v>0.31964092339757999</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>17</v>
       </c>
@@ -5074,7 +5074,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>34</v>
       </c>
@@ -5127,7 +5127,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>140</v>
       </c>
@@ -5180,7 +5180,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>41</v>
       </c>
@@ -5233,7 +5233,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>45</v>
       </c>
@@ -5339,7 +5339,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>17</v>
       </c>
@@ -5392,7 +5392,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>17</v>
       </c>
@@ -5498,7 +5498,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>17</v>
       </c>
@@ -5604,7 +5604,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>34</v>
       </c>
@@ -5657,7 +5657,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>34</v>
       </c>
@@ -5816,7 +5816,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>34</v>
       </c>
@@ -5922,7 +5922,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>140</v>
       </c>
@@ -5975,7 +5975,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>140</v>
       </c>
@@ -6081,7 +6081,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>140</v>
       </c>
@@ -6187,7 +6187,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>41</v>
       </c>
@@ -6240,7 +6240,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>41</v>
       </c>
@@ -6346,7 +6346,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>41</v>
       </c>
@@ -6452,7 +6452,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>45</v>
       </c>
@@ -6505,7 +6505,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>45</v>
       </c>
@@ -6611,7 +6611,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>45</v>
       </c>
@@ -6666,6 +6666,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:Q110" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="USHINDI BAR"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="11">
       <filters>
         <filter val="20.90672294"/>
@@ -6702,5 +6707,6 @@
     </filterColumn>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>